<commit_message>
feat: improve file actions
</commit_message>
<xml_diff>
--- a/pipeline/ExcelPipeline/MySheet.xlsx
+++ b/pipeline/ExcelPipeline/MySheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tomdraper\Documents\Development\excel-pipeline\pipeline\ExcelPipeline\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA679E80-ED3E-4A4E-8947-7399951D71CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED4B63AC-80C2-44E6-BDD6-01AA57DD7134}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <x:bookViews>
     <x:workbookView xWindow="330" yWindow="2490" windowWidth="21600" windowHeight="11610" firstSheet="0" activeTab="0" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </x:bookViews>
@@ -392,83 +392,83 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" spans="1:2" x14ac:dyDescent="0.25">
-      <x:c r="A1" s="0">
+      <x:c r="A1" s="0" t="s">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="B1" s="0">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="B1" s="0" t="s">
-        <x:v>0</x:v>
-      </x:c>
     </x:row>
     <x:row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <x:c r="A2" s="0">
+      <x:c r="A2" s="0" t="s">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B2" s="0">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="B2" s="0" t="s">
-        <x:v>1</x:v>
-      </x:c>
     </x:row>
     <x:row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <x:c r="A3" s="0">
+      <x:c r="A3" s="0" t="s">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B3" s="0">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="B3" s="0" t="s">
-        <x:v>2</x:v>
-      </x:c>
     </x:row>
     <x:row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <x:c r="A4" s="0">
+      <x:c r="A4" s="0" t="s">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B4" s="0">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="B4" s="0" t="s">
-        <x:v>3</x:v>
-      </x:c>
     </x:row>
     <x:row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <x:c r="A5" s="0">
+      <x:c r="A5" s="0" t="s">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B5" s="0">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="B5" s="0" t="s">
-        <x:v>4</x:v>
-      </x:c>
     </x:row>
     <x:row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <x:c r="A6" s="0">
+      <x:c r="A6" s="0" t="s">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B6" s="0">
         <x:v>6</x:v>
       </x:c>
-      <x:c r="B6" s="0" t="s">
-        <x:v>5</x:v>
-      </x:c>
     </x:row>
     <x:row r="7" spans="1:2" x14ac:dyDescent="0.25">
-      <x:c r="A7" s="0">
+      <x:c r="A7" s="0" t="s">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="B7" s="0">
         <x:v>7</x:v>
       </x:c>
-      <x:c r="B7" s="0" t="s">
-        <x:v>6</x:v>
-      </x:c>
     </x:row>
     <x:row r="8" spans="1:2" x14ac:dyDescent="0.25">
-      <x:c r="A8" s="0">
+      <x:c r="A8" s="0" t="s">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="B8" s="0">
         <x:v>8</x:v>
       </x:c>
-      <x:c r="B8" s="0" t="s">
-        <x:v>7</x:v>
-      </x:c>
     </x:row>
     <x:row r="9" spans="1:2" x14ac:dyDescent="0.25">
-      <x:c r="A9" s="0">
+      <x:c r="A9" s="0" t="s">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B9" s="0">
         <x:v>9</x:v>
       </x:c>
-      <x:c r="B9" s="0" t="s">
-        <x:v>8</x:v>
-      </x:c>
     </x:row>
     <x:row r="10" spans="1:2" x14ac:dyDescent="0.25">
-      <x:c r="A10" s="0">
+      <x:c r="A10" s="0" t="s">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="B10" s="0">
         <x:v>10</x:v>
-      </x:c>
-      <x:c r="B10" s="0" t="s">
-        <x:v>9</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>